<commit_message>
Add per-folder READMEs and pipeline guide; remove em dashes; plainer wording
</commit_message>
<xml_diff>
--- a/data/outputs/fmcg_newsletter_20260621.xlsx
+++ b/data/outputs/fmcg_newsletter_20260621.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -789,12 +789,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -964,7 +964,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0.9251</t>
+          <t>0.9229</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1058,7 +1058,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0.8505</t>
+          <t>0.8483</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1152,7 +1152,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0.7893</t>
+          <t>0.7871</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1242,7 +1242,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0.7666</t>
+          <t>0.7644</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1328,7 +1328,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0.755</t>
+          <t>0.7528</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1414,7 +1414,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0.754</t>
+          <t>0.7518</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1500,7 +1500,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0.738</t>
+          <t>0.7358</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1590,7 +1590,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0.7342</t>
+          <t>0.732</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1676,7 +1676,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0.7188</t>
+          <t>0.7166</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1766,7 +1766,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0.7157</t>
+          <t>0.7135</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1856,7 +1856,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0.7117</t>
+          <t>0.7095</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0.7064</t>
+          <t>0.7042</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2032,7 +2032,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0.7018</t>
+          <t>0.6996</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2118,7 +2118,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0.6722</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2208,7 +2208,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0.6578</t>
+          <t>0.6556</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2294,7 +2294,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0.6546</t>
+          <t>0.6524</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2380,7 +2380,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0.6478</t>
+          <t>0.6456</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2470,7 +2470,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.6377</t>
+          <t>0.6355</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2556,7 +2556,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.5905</t>
+          <t>0.5883</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2642,7 +2642,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.5847</t>
+          <t>0.5825</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2728,7 +2728,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.4871</t>
+          <t>0.4849</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2818,7 +2818,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.4778</t>
+          <t>0.4756</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2900,7 +2900,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.4593</t>
+          <t>0.4571</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2982,7 +2982,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0.3687</t>
+          <t>0.3665</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3060,7 +3060,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0.3364</t>
+          <t>0.3342</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3170,49 +3170,49 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Ingestion: public RSS/Atom feeds (Google News deal queries + FMCG trade press), filtered to the last 14 days. No paywalled or private sources.</t>
+          <t>Ingestion: public RSS/Atom feeds (Google News + FMCG trade press), last 14 days.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>De-duplication: exact match on normalised URL/title, then near-duplicate clustering. Each story is fingerprinted by its named entities (companies, brands) and figures plus significant content words; two reports merge when they share at least 2 entities AND their blended overlap (entity + content overlap coefficients) reaches 0.50. The most credible/recent report is kept as the representative. 5 of 30 articles merged this run.</t>
+          <t>De-duplication: exact URL/title match, then near-dup clustering by entity overlap (threshold 0.5). 5 of 30 articles merged.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Relevance: an item must show BOTH a deal signal (acquire/merger/stake/funding…) and an FMCG signal (category or named consumer-goods company); title matches weighted x2. Items scoring below 35/100 are dropped from the draft.</t>
+          <t>Relevance: requires a deal signal AND an FMCG signal (title ×2). Items below 35/100 are dropped.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Credibility: transparent source-tier allow-list (global wire &gt; trade press &gt; general &gt; press-release wires), plus a corroboration bonus when multiple independent outlets report the same deal, and a penalty for lone press releases. We rate the SOURCE, not each claim.</t>
+          <t>Credibility: source-tier allow-list + corroboration bonus − lone press-release penalty.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Ranking: composite of relevance (45%), credibility (30%), recency (15%) and corroboration (10%).</t>
+          <t>Ranking: relevance 45%, credibility 30%, recency 15%, corroboration 10%.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Summaries: template-generated from extracted deal facts + the source blurb (no LLM key set).</t>
+          <t>Summaries: template from extracted deal facts + source blurb (no LLM_API_KEY set).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Assumptions &amp; limits: deal value/parties are extracted heuristically (regex) and may be incomplete; coverage reflects what public feeds surface; this is decision-support, not advice.</t>
+          <t>Deal value/parties are regex heuristics and may be incomplete. Decision-support only.</t>
         </is>
       </c>
     </row>

</xml_diff>